<commit_message>
CORRECTED PROV_TOT and re-knit all global
</commit_message>
<xml_diff>
--- a/Extracted_data_analysis/global/Output-Transformed_data/geographical_distribution_summary.xlsx
+++ b/Extracted_data_analysis/global/Output-Transformed_data/geographical_distribution_summary.xlsx
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>420</v>
+        <v>330</v>
       </c>
     </row>
     <row r="5">
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>389</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>91</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>272</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19">
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="B20">
-        <v>173</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>58</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="B41">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -1123,7 +1123,7 @@
         </is>
       </c>
       <c r="B51">
-        <v>49</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1133,7 +1133,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1160,10 +1160,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>446</v>
+        <v>955</v>
       </c>
       <c r="C2">
-        <v>45</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -1173,10 +1173,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>168</v>
+        <v>40</v>
       </c>
       <c r="C3">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1186,10 +1186,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>349</v>
+        <v>4</v>
       </c>
       <c r="C4">
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1199,87 +1199,22 @@
         </is>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B6">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>15</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>1</v>
-      </c>
-      <c r="C11">
         <v>0</v>
       </c>
     </row>

</xml_diff>